<commit_message>
Rename the attachment's sheets to CPI / Offshore / FATF, and 辖区 → 国家/地区
Legal asked for uniform sheet names and for the offshore and FATF sheets to label
their entries the way CPI already does. Two things had to move with them:

- the upload backend and load_baseline matched the FATF sheet by one exact string,
  so they now match any sheet whose name starts with FATF. A workbook Legal saved
  before this change still uploads.
- the CPI edition year came from the sheet title ("CPI 2025"). With the title now
  just "CPI" it falls back to the year in the row-1 note — losing it would have
  silently disabled the edition comparison that decides whether the override or
  the fetch wins.

The seed baseline workbook is renamed to match, since Legal edits that file too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/data-refresh/seeds/fatf-baseline.xlsx
+++ b/scripts/data-refresh/seeds/fatf-baseline.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPI 2025" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offshore Centres 离岸中心" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FATF 黑灰名单" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offshore" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FATF" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3498,7 +3498,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>辖区 Jurisdiction</t>
+          <t>国家/地区 Country</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>辖区 Jurisdiction</t>
+          <t>国家/地区 Country</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add an ISO 3166-1 alpha-2 code column beside every country name
Alpha-2 rather than alpha-3 because it is the code the rest of the pipeline already
speaks: SAP's vendor_master.land1 is a 2-char country key and D&B returns
countryISOAlpha2Code, so these lists now join onto our own data without matching on
names.

Codes come from seeds/iso3166.json, generated by build_iso3166_seed.py from the
public-domain zoneinfo table plus the codes the offshore fetcher already resolves;
the generator exits non-zero if any country in the three snapshots fails to resolve,
and all 247 rows currently resolve. The table is committed so CI does not depend on
a file being present on the runner.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/data-refresh/seeds/fatf-baseline.xlsx
+++ b/scripts/data-refresh/seeds/fatf-baseline.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +115,12 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,12 +486,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D184"/>
+  <dimension ref="A1:E184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -507,12 +513,17 @@
           <t>国家/地区 Country</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>代码 Code</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>分数 Score</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>≤/&gt; 阈值40</t>
         </is>
@@ -527,10 +538,15 @@
           <t>Denmark</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
         <v>89</v>
       </c>
-      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -541,10 +557,15 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>FI</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -555,10 +576,15 @@
           <t>Singapore</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>84</v>
       </c>
-      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -569,10 +595,15 @@
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>NZ</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>81</v>
       </c>
-      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -583,10 +614,15 @@
           <t>Norway</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>81</v>
       </c>
-      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -597,10 +633,15 @@
           <t>Sweden</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -611,10 +652,15 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -625,10 +671,15 @@
           <t>Luxembourg</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>LU</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
         <v>78</v>
       </c>
-      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -639,10 +690,15 @@
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
         <v>78</v>
       </c>
-      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -653,10 +709,15 @@
           <t>Germany</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
         <v>77</v>
       </c>
-      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -667,10 +728,15 @@
           <t>Iceland</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
         <v>77</v>
       </c>
-      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -681,10 +747,15 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -695,10 +766,15 @@
           <t>Estonia</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>EE</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -709,10 +785,15 @@
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -723,10 +804,15 @@
           <t>Ireland</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -737,10 +823,15 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -751,10 +842,15 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>UY</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -765,10 +861,15 @@
           <t>Bhutan</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>BT</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -779,10 +880,15 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -793,10 +899,15 @@
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -807,10 +918,15 @@
           <t>Austria</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -821,10 +937,15 @@
           <t>Belgium</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -835,10 +956,15 @@
           <t>United Arab Emirates</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -849,10 +975,15 @@
           <t>Barbados</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n">
         <v>68</v>
       </c>
-      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -863,10 +994,15 @@
           <t>Seychelles</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="n">
         <v>68</v>
       </c>
-      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -877,10 +1013,15 @@
           <t>Taiwan</t>
         </is>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="n">
         <v>68</v>
       </c>
-      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -891,10 +1032,15 @@
           <t>France</t>
         </is>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="n">
         <v>66</v>
       </c>
-      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -905,10 +1051,15 @@
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -919,10 +1070,15 @@
           <t>Bahamas</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>BS</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -933,10 +1089,15 @@
           <t>United States of America</t>
         </is>
       </c>
-      <c r="C32" s="4" t="n">
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -947,10 +1108,15 @@
           <t>Brunei Darussalam</t>
         </is>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>BN</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -961,10 +1127,15 @@
           <t>Chile</t>
         </is>
       </c>
-      <c r="C34" s="4" t="n">
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="D34" s="5" t="n"/>
+      <c r="E34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -975,10 +1146,15 @@
           <t>Korea, South</t>
         </is>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -989,10 +1165,15 @@
           <t>Saint Vincent and the Grenadines</t>
         </is>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="D36" s="5" t="n"/>
+      <c r="E36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -1003,10 +1184,15 @@
           <t>Cabo Verde</t>
         </is>
       </c>
-      <c r="C37" s="4" t="n">
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>CV</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -1017,10 +1203,15 @@
           <t>Israel</t>
         </is>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -1031,10 +1222,15 @@
           <t>Dominica</t>
         </is>
       </c>
-      <c r="C39" s="4" t="n">
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -1045,10 +1241,15 @@
           <t>Latvia</t>
         </is>
       </c>
-      <c r="C40" s="4" t="n">
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -1059,10 +1260,15 @@
           <t>Czechia</t>
         </is>
       </c>
-      <c r="C41" s="4" t="n">
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
@@ -1073,10 +1279,15 @@
           <t>Saint Lucia</t>
         </is>
       </c>
-      <c r="C42" s="4" t="n">
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>LC</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="D42" s="5" t="n"/>
+      <c r="E42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -1087,10 +1298,15 @@
           <t>Botswana</t>
         </is>
       </c>
-      <c r="C43" s="4" t="n">
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="D43" s="5" t="n"/>
+      <c r="E43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -1101,10 +1317,15 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C44" s="4" t="n">
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -1115,10 +1336,15 @@
           <t>Rwanda</t>
         </is>
       </c>
-      <c r="C45" s="4" t="n">
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -1129,10 +1355,15 @@
           <t>Slovenia</t>
         </is>
       </c>
-      <c r="C46" s="4" t="n">
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="D46" s="5" t="n"/>
+      <c r="E46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -1143,10 +1374,15 @@
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="C47" s="4" t="n">
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="n">
         <v>57</v>
       </c>
-      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -1157,10 +1393,15 @@
           <t>Costa Rica</t>
         </is>
       </c>
-      <c r="C48" s="4" t="n">
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -1171,10 +1412,15 @@
           <t>Grenada</t>
         </is>
       </c>
-      <c r="C49" s="4" t="n">
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
@@ -1185,10 +1431,15 @@
           <t>Portugal</t>
         </is>
       </c>
-      <c r="C50" s="4" t="n">
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="D50" s="5" t="n"/>
+      <c r="E50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -1199,10 +1450,15 @@
           <t>Cyprus</t>
         </is>
       </c>
-      <c r="C51" s="4" t="n">
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>CY</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -1213,10 +1469,15 @@
           <t>Fiji</t>
         </is>
       </c>
-      <c r="C52" s="4" t="n">
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>FJ</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="D52" s="5" t="n"/>
+      <c r="E52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -1227,10 +1488,15 @@
           <t>Spain</t>
         </is>
       </c>
-      <c r="C53" s="4" t="n">
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="D53" s="5" t="n"/>
+      <c r="E53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -1241,10 +1507,15 @@
           <t>Italy</t>
         </is>
       </c>
-      <c r="C54" s="4" t="n">
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="D54" s="5" t="n"/>
+      <c r="E54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -1255,10 +1526,15 @@
           <t>Poland</t>
         </is>
       </c>
-      <c r="C55" s="4" t="n">
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="D55" s="5" t="n"/>
+      <c r="E55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
@@ -1269,10 +1545,15 @@
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="C56" s="4" t="n">
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="D56" s="5" t="n"/>
+      <c r="E56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -1283,10 +1564,15 @@
           <t>Oman</t>
         </is>
       </c>
-      <c r="C57" s="4" t="n">
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>OM</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="D57" s="5" t="n"/>
+      <c r="E57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n">
@@ -1297,10 +1583,15 @@
           <t>Bahrain</t>
         </is>
       </c>
-      <c r="C58" s="4" t="n">
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>BH</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D58" s="5" t="n"/>
+      <c r="E58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -1311,10 +1602,15 @@
           <t>Georgia</t>
         </is>
       </c>
-      <c r="C59" s="4" t="n">
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>GE</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D59" s="5" t="n"/>
+      <c r="E59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">
@@ -1325,10 +1621,15 @@
           <t>Greece</t>
         </is>
       </c>
-      <c r="C60" s="4" t="n">
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D60" s="5" t="n"/>
+      <c r="E60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -1339,10 +1640,15 @@
           <t>Jordan</t>
         </is>
       </c>
-      <c r="C61" s="4" t="n">
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>JO</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D61" s="5" t="n"/>
+      <c r="E61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n">
@@ -1353,10 +1659,15 @@
           <t>Malta</t>
         </is>
       </c>
-      <c r="C62" s="4" t="n">
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D62" s="5" t="n"/>
+      <c r="E62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
@@ -1367,10 +1678,15 @@
           <t>Mauritius</t>
         </is>
       </c>
-      <c r="C63" s="4" t="n">
+      <c r="C63" s="11" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="D63" s="5" t="n"/>
+      <c r="E63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
@@ -1381,10 +1697,15 @@
           <t>Slovakia</t>
         </is>
       </c>
-      <c r="C64" s="4" t="n">
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>SK</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="D64" s="5" t="n"/>
+      <c r="E64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
@@ -1395,10 +1716,15 @@
           <t>Croatia</t>
         </is>
       </c>
-      <c r="C65" s="4" t="n">
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="D65" s="5" t="n"/>
+      <c r="E65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n">
@@ -1409,10 +1735,15 @@
           <t>Vanuatu</t>
         </is>
       </c>
-      <c r="C66" s="4" t="n">
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>VU</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n">
@@ -1423,10 +1754,15 @@
           <t>Armenia</t>
         </is>
       </c>
-      <c r="C67" s="4" t="n">
+      <c r="C67" s="11" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="D67" s="5" t="n"/>
+      <c r="E67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n">
@@ -1437,10 +1773,15 @@
           <t>Kuwait</t>
         </is>
       </c>
-      <c r="C68" s="4" t="n">
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="D68" s="5" t="n"/>
+      <c r="E68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n">
@@ -1451,10 +1792,15 @@
           <t>Montenegro</t>
         </is>
       </c>
-      <c r="C69" s="4" t="n">
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="D69" s="5" t="n"/>
+      <c r="E69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n">
@@ -1465,10 +1811,15 @@
           <t>Namibia</t>
         </is>
       </c>
-      <c r="C70" s="4" t="n">
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="D70" s="5" t="n"/>
+      <c r="E70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
@@ -1479,10 +1830,15 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="C71" s="4" t="n">
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="D71" s="5" t="n"/>
+      <c r="E71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n">
@@ -1493,10 +1849,15 @@
           <t>Benin</t>
         </is>
       </c>
-      <c r="C72" s="4" t="n">
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>BJ</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="D72" s="5" t="n"/>
+      <c r="E72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n">
@@ -1507,10 +1868,15 @@
           <t>Romania</t>
         </is>
       </c>
-      <c r="C73" s="4" t="n">
+      <c r="C73" s="11" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="D73" s="5" t="n"/>
+      <c r="E73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n">
@@ -1521,10 +1887,15 @@
           <t>Sao Tome and Principe</t>
         </is>
       </c>
-      <c r="C74" s="4" t="n">
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="D74" s="5" t="n"/>
+      <c r="E74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n">
@@ -1535,10 +1906,15 @@
           <t>Jamaica</t>
         </is>
       </c>
-      <c r="C75" s="4" t="n">
+      <c r="C75" s="11" t="inlineStr">
+        <is>
+          <t>JM</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="D75" s="5" t="n"/>
+      <c r="E75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n">
@@ -1549,10 +1925,15 @@
           <t>Solomon Islands</t>
         </is>
       </c>
-      <c r="C76" s="4" t="n">
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>SB</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="D76" s="5" t="n"/>
+      <c r="E76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
@@ -1563,10 +1944,15 @@
           <t>Timor-Leste</t>
         </is>
       </c>
-      <c r="C77" s="4" t="n">
+      <c r="C77" s="11" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="D77" s="5" t="n"/>
+      <c r="E77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n">
@@ -1577,10 +1963,15 @@
           <t>China</t>
         </is>
       </c>
-      <c r="C78" s="4" t="n">
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="D78" s="5" t="n"/>
+      <c r="E78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
@@ -1591,10 +1982,15 @@
           <t>Cote d'Ivoire</t>
         </is>
       </c>
-      <c r="C79" s="4" t="n">
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="D79" s="5" t="n"/>
+      <c r="E79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n">
@@ -1605,10 +2001,15 @@
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C80" s="4" t="n">
+      <c r="C80" s="11" t="inlineStr">
+        <is>
+          <t>GH</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="D80" s="5" t="n"/>
+      <c r="E80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
@@ -1619,10 +2020,15 @@
           <t>Kosovo</t>
         </is>
       </c>
-      <c r="C81" s="4" t="n">
+      <c r="C81" s="11" t="inlineStr">
+        <is>
+          <t>XK</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="D81" s="5" t="n"/>
+      <c r="E81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -1633,10 +2039,15 @@
           <t>Moldova</t>
         </is>
       </c>
-      <c r="C82" s="4" t="n">
+      <c r="C82" s="11" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="D82" s="5" t="n"/>
+      <c r="E82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
@@ -1647,10 +2058,15 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="C83" s="4" t="n">
+      <c r="C83" s="11" t="inlineStr">
+        <is>
+          <t>ZA</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="D83" s="5" t="n"/>
+      <c r="E83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n">
@@ -1661,10 +2077,15 @@
           <t>Trinidad and Tobago</t>
         </is>
       </c>
-      <c r="C84" s="4" t="n">
+      <c r="C84" s="11" t="inlineStr">
+        <is>
+          <t>TT</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="D84" s="5" t="n"/>
+      <c r="E84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -1675,10 +2096,15 @@
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C85" s="4" t="n">
+      <c r="C85" s="11" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="D85" s="5" t="n"/>
+      <c r="E85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="6" t="n">
@@ -1689,10 +2115,15 @@
           <t>Bulgaria</t>
         </is>
       </c>
-      <c r="C86" s="6" t="n">
+      <c r="C86" s="11" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="D86" s="7" t="inlineStr">
+      <c r="E86" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1707,10 +2138,15 @@
           <t>Burkina Faso</t>
         </is>
       </c>
-      <c r="C87" s="6" t="n">
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="D87" s="7" t="inlineStr">
+      <c r="E87" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1725,10 +2161,15 @@
           <t>Cuba</t>
         </is>
       </c>
-      <c r="C88" s="6" t="n">
+      <c r="C88" s="11" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="D88" s="7" t="inlineStr">
+      <c r="E88" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1743,10 +2184,15 @@
           <t>Guyana</t>
         </is>
       </c>
-      <c r="C89" s="6" t="n">
+      <c r="C89" s="11" t="inlineStr">
+        <is>
+          <t>GY</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="D89" s="7" t="inlineStr">
+      <c r="E89" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1761,10 +2207,15 @@
           <t>Hungary</t>
         </is>
       </c>
-      <c r="C90" s="6" t="n">
+      <c r="C90" s="11" t="inlineStr">
+        <is>
+          <t>HU</t>
+        </is>
+      </c>
+      <c r="D90" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="D90" s="7" t="inlineStr">
+      <c r="E90" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1779,10 +2230,15 @@
           <t>North Macedonia</t>
         </is>
       </c>
-      <c r="C91" s="6" t="n">
+      <c r="C91" s="11" t="inlineStr">
+        <is>
+          <t>MK</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="E91" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1797,10 +2253,15 @@
           <t>Tanzania</t>
         </is>
       </c>
-      <c r="C92" s="6" t="n">
+      <c r="C92" s="11" t="inlineStr">
+        <is>
+          <t>TZ</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="D92" s="7" t="inlineStr">
+      <c r="E92" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1815,10 +2276,15 @@
           <t>Albania</t>
         </is>
       </c>
-      <c r="C93" s="6" t="n">
+      <c r="C93" s="11" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="D93" s="7" t="inlineStr">
+      <c r="E93" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1833,10 +2299,15 @@
           <t>India</t>
         </is>
       </c>
-      <c r="C94" s="6" t="n">
+      <c r="C94" s="11" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D94" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="D94" s="7" t="inlineStr">
+      <c r="E94" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1851,10 +2322,15 @@
           <t>Maldives</t>
         </is>
       </c>
-      <c r="C95" s="6" t="n">
+      <c r="C95" s="11" t="inlineStr">
+        <is>
+          <t>MV</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="D95" s="7" t="inlineStr">
+      <c r="E95" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1869,10 +2345,15 @@
           <t>Morocco</t>
         </is>
       </c>
-      <c r="C96" s="6" t="n">
+      <c r="C96" s="11" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D96" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="E96" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1887,10 +2368,15 @@
           <t>Tunisia</t>
         </is>
       </c>
-      <c r="C97" s="6" t="n">
+      <c r="C97" s="11" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="D97" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="D97" s="7" t="inlineStr">
+      <c r="E97" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1905,10 +2391,15 @@
           <t>Ethiopia</t>
         </is>
       </c>
-      <c r="C98" s="6" t="n">
+      <c r="C98" s="11" t="inlineStr">
+        <is>
+          <t>ET</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="D98" s="7" t="inlineStr">
+      <c r="E98" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1923,10 +2414,15 @@
           <t>Kazakhstan</t>
         </is>
       </c>
-      <c r="C99" s="6" t="n">
+      <c r="C99" s="11" t="inlineStr">
+        <is>
+          <t>KZ</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="D99" s="7" t="inlineStr">
+      <c r="E99" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1941,10 +2437,15 @@
           <t>Suriname</t>
         </is>
       </c>
-      <c r="C100" s="6" t="n">
+      <c r="C100" s="11" t="inlineStr">
+        <is>
+          <t>SR</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="D100" s="7" t="inlineStr">
+      <c r="E100" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1959,10 +2460,15 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="C101" s="6" t="n">
+      <c r="C101" s="11" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="D101" s="7" t="inlineStr">
+      <c r="E101" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1977,10 +2483,15 @@
           <t>Dominican Republic</t>
         </is>
       </c>
-      <c r="C102" s="6" t="n">
+      <c r="C102" s="11" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="D102" s="7" t="inlineStr">
+      <c r="E102" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -1995,10 +2506,15 @@
           <t>Gambia</t>
         </is>
       </c>
-      <c r="C103" s="6" t="n">
+      <c r="C103" s="11" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="D103" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="D103" s="7" t="inlineStr">
+      <c r="E103" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2013,10 +2529,15 @@
           <t>Lesotho</t>
         </is>
       </c>
-      <c r="C104" s="6" t="n">
+      <c r="C104" s="11" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="D104" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="D104" s="7" t="inlineStr">
+      <c r="E104" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2031,10 +2552,15 @@
           <t>Zambia</t>
         </is>
       </c>
-      <c r="C105" s="6" t="n">
+      <c r="C105" s="11" t="inlineStr">
+        <is>
+          <t>ZM</t>
+        </is>
+      </c>
+      <c r="D105" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="D105" s="7" t="inlineStr">
+      <c r="E105" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2049,10 +2575,15 @@
           <t>Argentina</t>
         </is>
       </c>
-      <c r="C106" s="6" t="n">
+      <c r="C106" s="11" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="D106" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="D106" s="7" t="inlineStr">
+      <c r="E106" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2067,10 +2598,15 @@
           <t>Belize</t>
         </is>
       </c>
-      <c r="C107" s="6" t="n">
+      <c r="C107" s="11" t="inlineStr">
+        <is>
+          <t>BZ</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="D107" s="7" t="inlineStr">
+      <c r="E107" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2085,10 +2621,15 @@
           <t>Ukraine</t>
         </is>
       </c>
-      <c r="C108" s="6" t="n">
+      <c r="C108" s="11" t="inlineStr">
+        <is>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="D108" s="7" t="inlineStr">
+      <c r="E108" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2103,10 +2644,15 @@
           <t>Brazil</t>
         </is>
       </c>
-      <c r="C109" s="6" t="n">
+      <c r="C109" s="11" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="D109" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="D109" s="7" t="inlineStr">
+      <c r="E109" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2121,10 +2667,15 @@
           <t>Sri Lanka</t>
         </is>
       </c>
-      <c r="C110" s="6" t="n">
+      <c r="C110" s="11" t="inlineStr">
+        <is>
+          <t>LK</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="D110" s="7" t="inlineStr">
+      <c r="E110" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2139,10 +2690,15 @@
           <t>Algeria</t>
         </is>
       </c>
-      <c r="C111" s="6" t="n">
+      <c r="C111" s="11" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="D111" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="D111" s="7" t="inlineStr">
+      <c r="E111" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2157,10 +2713,15 @@
           <t>Bosnia and Herzegovina</t>
         </is>
       </c>
-      <c r="C112" s="6" t="n">
+      <c r="C112" s="11" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="D112" s="7" t="inlineStr">
+      <c r="E112" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2175,10 +2736,15 @@
           <t>Indonesia</t>
         </is>
       </c>
-      <c r="C113" s="6" t="n">
+      <c r="C113" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="D113" s="7" t="inlineStr">
+      <c r="E113" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2193,10 +2759,15 @@
           <t>Laos</t>
         </is>
       </c>
-      <c r="C114" s="6" t="n">
+      <c r="C114" s="11" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="D114" s="7" t="inlineStr">
+      <c r="E114" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2211,10 +2782,15 @@
           <t>Malawi</t>
         </is>
       </c>
-      <c r="C115" s="6" t="n">
+      <c r="C115" s="11" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="D115" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="D115" s="7" t="inlineStr">
+      <c r="E115" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2229,10 +2805,15 @@
           <t>Nepal</t>
         </is>
       </c>
-      <c r="C116" s="6" t="n">
+      <c r="C116" s="11" t="inlineStr">
+        <is>
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="D116" s="7" t="inlineStr">
+      <c r="E116" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2247,10 +2828,15 @@
           <t>Sierra Leone</t>
         </is>
       </c>
-      <c r="C117" s="6" t="n">
+      <c r="C117" s="11" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="D117" s="7" t="inlineStr">
+      <c r="E117" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2265,10 +2851,15 @@
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="C118" s="6" t="n">
+      <c r="C118" s="11" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="D118" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="D118" s="7" t="inlineStr">
+      <c r="E118" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2283,10 +2874,15 @@
           <t>Panama</t>
         </is>
       </c>
-      <c r="C119" s="6" t="n">
+      <c r="C119" s="11" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="D119" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="D119" s="7" t="inlineStr">
+      <c r="E119" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2301,10 +2897,15 @@
           <t>Serbia</t>
         </is>
       </c>
-      <c r="C120" s="6" t="n">
+      <c r="C120" s="11" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="D120" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="D120" s="7" t="inlineStr">
+      <c r="E120" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2319,10 +2920,15 @@
           <t>Thailand</t>
         </is>
       </c>
-      <c r="C121" s="6" t="n">
+      <c r="C121" s="11" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D121" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="D121" s="7" t="inlineStr">
+      <c r="E121" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2337,10 +2943,15 @@
           <t>Angola</t>
         </is>
       </c>
-      <c r="C122" s="6" t="n">
+      <c r="C122" s="11" t="inlineStr">
+        <is>
+          <t>AO</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="D122" s="7" t="inlineStr">
+      <c r="E122" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2355,10 +2966,15 @@
           <t>El Salvador</t>
         </is>
       </c>
-      <c r="C123" s="6" t="n">
+      <c r="C123" s="11" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="D123" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="D123" s="7" t="inlineStr">
+      <c r="E123" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2373,10 +2989,15 @@
           <t>Philippines</t>
         </is>
       </c>
-      <c r="C124" s="6" t="n">
+      <c r="C124" s="11" t="inlineStr">
+        <is>
+          <t>PH</t>
+        </is>
+      </c>
+      <c r="D124" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="D124" s="7" t="inlineStr">
+      <c r="E124" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2391,10 +3012,15 @@
           <t>Togo</t>
         </is>
       </c>
-      <c r="C125" s="6" t="n">
+      <c r="C125" s="11" t="inlineStr">
+        <is>
+          <t>TG</t>
+        </is>
+      </c>
+      <c r="D125" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="D125" s="7" t="inlineStr">
+      <c r="E125" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2409,10 +3035,15 @@
           <t>Belarus</t>
         </is>
       </c>
-      <c r="C126" s="6" t="n">
+      <c r="C126" s="11" t="inlineStr">
+        <is>
+          <t>BY</t>
+        </is>
+      </c>
+      <c r="D126" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="D126" s="7" t="inlineStr">
+      <c r="E126" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2427,10 +3058,15 @@
           <t>Djibouti</t>
         </is>
       </c>
-      <c r="C127" s="6" t="n">
+      <c r="C127" s="11" t="inlineStr">
+        <is>
+          <t>DJ</t>
+        </is>
+      </c>
+      <c r="D127" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="D127" s="7" t="inlineStr">
+      <c r="E127" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2445,10 +3081,15 @@
           <t>Mongolia</t>
         </is>
       </c>
-      <c r="C128" s="6" t="n">
+      <c r="C128" s="11" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="D128" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="D128" s="7" t="inlineStr">
+      <c r="E128" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2463,10 +3104,15 @@
           <t>Niger</t>
         </is>
       </c>
-      <c r="C129" s="6" t="n">
+      <c r="C129" s="11" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="D129" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="D129" s="7" t="inlineStr">
+      <c r="E129" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2481,10 +3127,15 @@
           <t>Turkey</t>
         </is>
       </c>
-      <c r="C130" s="6" t="n">
+      <c r="C130" s="11" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="D130" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="D130" s="7" t="inlineStr">
+      <c r="E130" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2499,10 +3150,15 @@
           <t>Uzbekistan</t>
         </is>
       </c>
-      <c r="C131" s="6" t="n">
+      <c r="C131" s="11" t="inlineStr">
+        <is>
+          <t>UZ</t>
+        </is>
+      </c>
+      <c r="D131" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="D131" s="7" t="inlineStr">
+      <c r="E131" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2517,10 +3173,15 @@
           <t>Azerbaijan</t>
         </is>
       </c>
-      <c r="C132" s="6" t="n">
+      <c r="C132" s="11" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="D132" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="D132" s="7" t="inlineStr">
+      <c r="E132" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2535,10 +3196,15 @@
           <t>Egypt</t>
         </is>
       </c>
-      <c r="C133" s="6" t="n">
+      <c r="C133" s="11" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="D133" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="D133" s="7" t="inlineStr">
+      <c r="E133" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2553,10 +3219,15 @@
           <t>Kenya</t>
         </is>
       </c>
-      <c r="C134" s="6" t="n">
+      <c r="C134" s="11" t="inlineStr">
+        <is>
+          <t>KE</t>
+        </is>
+      </c>
+      <c r="D134" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="D134" s="7" t="inlineStr">
+      <c r="E134" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2571,10 +3242,15 @@
           <t>Mauritania</t>
         </is>
       </c>
-      <c r="C135" s="6" t="n">
+      <c r="C135" s="11" t="inlineStr">
+        <is>
+          <t>MR</t>
+        </is>
+      </c>
+      <c r="D135" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="D135" s="7" t="inlineStr">
+      <c r="E135" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2589,10 +3265,15 @@
           <t>Peru</t>
         </is>
       </c>
-      <c r="C136" s="6" t="n">
+      <c r="C136" s="11" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="D136" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="D136" s="7" t="inlineStr">
+      <c r="E136" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2607,10 +3288,15 @@
           <t>Gabon</t>
         </is>
       </c>
-      <c r="C137" s="6" t="n">
+      <c r="C137" s="11" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D137" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="D137" s="7" t="inlineStr">
+      <c r="E137" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2625,10 +3311,15 @@
           <t>Bolivia</t>
         </is>
       </c>
-      <c r="C138" s="6" t="n">
+      <c r="C138" s="11" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="D138" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="D138" s="7" t="inlineStr">
+      <c r="E138" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2643,10 +3334,15 @@
           <t>Iraq</t>
         </is>
       </c>
-      <c r="C139" s="6" t="n">
+      <c r="C139" s="11" t="inlineStr">
+        <is>
+          <t>IQ</t>
+        </is>
+      </c>
+      <c r="D139" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="D139" s="7" t="inlineStr">
+      <c r="E139" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2661,10 +3357,15 @@
           <t>Liberia</t>
         </is>
       </c>
-      <c r="C140" s="6" t="n">
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="D140" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="D140" s="7" t="inlineStr">
+      <c r="E140" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2679,10 +3380,15 @@
           <t>Mali</t>
         </is>
       </c>
-      <c r="C141" s="6" t="n">
+      <c r="C141" s="11" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="D141" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="D141" s="7" t="inlineStr">
+      <c r="E141" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2697,10 +3403,15 @@
           <t>Pakistan</t>
         </is>
       </c>
-      <c r="C142" s="6" t="n">
+      <c r="C142" s="11" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="D142" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="D142" s="7" t="inlineStr">
+      <c r="E142" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2715,10 +3426,15 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="C143" s="6" t="n">
+      <c r="C143" s="11" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="D143" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="D143" s="7" t="inlineStr">
+      <c r="E143" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2733,10 +3449,15 @@
           <t>Cameroon</t>
         </is>
       </c>
-      <c r="C144" s="6" t="n">
+      <c r="C144" s="11" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="D144" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="D144" s="7" t="inlineStr">
+      <c r="E144" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2751,10 +3472,15 @@
           <t>Guatemala</t>
         </is>
       </c>
-      <c r="C145" s="6" t="n">
+      <c r="C145" s="11" t="inlineStr">
+        <is>
+          <t>GT</t>
+        </is>
+      </c>
+      <c r="D145" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="D145" s="7" t="inlineStr">
+      <c r="E145" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2769,10 +3495,15 @@
           <t>Guinea</t>
         </is>
       </c>
-      <c r="C146" s="6" t="n">
+      <c r="C146" s="11" t="inlineStr">
+        <is>
+          <t>GN</t>
+        </is>
+      </c>
+      <c r="D146" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="D146" s="7" t="inlineStr">
+      <c r="E146" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2787,10 +3518,15 @@
           <t>Kyrgyzstan</t>
         </is>
       </c>
-      <c r="C147" s="6" t="n">
+      <c r="C147" s="11" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D147" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="D147" s="7" t="inlineStr">
+      <c r="E147" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2805,10 +3541,15 @@
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C148" s="6" t="n">
+      <c r="C148" s="11" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D148" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="D148" s="7" t="inlineStr">
+      <c r="E148" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2823,10 +3564,15 @@
           <t>Papua New Guinea</t>
         </is>
       </c>
-      <c r="C149" s="6" t="n">
+      <c r="C149" s="11" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D149" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="D149" s="7" t="inlineStr">
+      <c r="E149" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2841,10 +3587,15 @@
           <t>Madagascar</t>
         </is>
       </c>
-      <c r="C150" s="6" t="n">
+      <c r="C150" s="11" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D150" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="D150" s="7" t="inlineStr">
+      <c r="E150" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2859,10 +3610,15 @@
           <t>Uganda</t>
         </is>
       </c>
-      <c r="C151" s="6" t="n">
+      <c r="C151" s="11" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+      <c r="D151" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="D151" s="7" t="inlineStr">
+      <c r="E151" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2877,10 +3633,15 @@
           <t>Bangladesh</t>
         </is>
       </c>
-      <c r="C152" s="6" t="n">
+      <c r="C152" s="11" t="inlineStr">
+        <is>
+          <t>BD</t>
+        </is>
+      </c>
+      <c r="D152" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="D152" s="7" t="inlineStr">
+      <c r="E152" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2895,10 +3656,15 @@
           <t>Central African Republic</t>
         </is>
       </c>
-      <c r="C153" s="6" t="n">
+      <c r="C153" s="11" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="D153" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="D153" s="7" t="inlineStr">
+      <c r="E153" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2913,10 +3679,15 @@
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="C154" s="6" t="n">
+      <c r="C154" s="11" t="inlineStr">
+        <is>
+          <t>PY</t>
+        </is>
+      </c>
+      <c r="D154" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="D154" s="7" t="inlineStr">
+      <c r="E154" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2931,10 +3702,15 @@
           <t>Congo</t>
         </is>
       </c>
-      <c r="C155" s="6" t="n">
+      <c r="C155" s="11" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="D155" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="D155" s="7" t="inlineStr">
+      <c r="E155" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2949,10 +3725,15 @@
           <t>Eswatini</t>
         </is>
       </c>
-      <c r="C156" s="6" t="n">
+      <c r="C156" s="11" t="inlineStr">
+        <is>
+          <t>SZ</t>
+        </is>
+      </c>
+      <c r="D156" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="D156" s="7" t="inlineStr">
+      <c r="E156" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2967,10 +3748,15 @@
           <t>Iran</t>
         </is>
       </c>
-      <c r="C157" s="6" t="n">
+      <c r="C157" s="11" t="inlineStr">
+        <is>
+          <t>IR</t>
+        </is>
+      </c>
+      <c r="D157" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="D157" s="7" t="inlineStr">
+      <c r="E157" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -2985,10 +3771,15 @@
           <t>Lebanon</t>
         </is>
       </c>
-      <c r="C158" s="6" t="n">
+      <c r="C158" s="11" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="D158" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="D158" s="7" t="inlineStr">
+      <c r="E158" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3003,10 +3794,15 @@
           <t>Chad</t>
         </is>
       </c>
-      <c r="C159" s="6" t="n">
+      <c r="C159" s="11" t="inlineStr">
+        <is>
+          <t>TD</t>
+        </is>
+      </c>
+      <c r="D159" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="D159" s="7" t="inlineStr">
+      <c r="E159" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3021,10 +3817,15 @@
           <t>Honduras</t>
         </is>
       </c>
-      <c r="C160" s="6" t="n">
+      <c r="C160" s="11" t="inlineStr">
+        <is>
+          <t>HN</t>
+        </is>
+      </c>
+      <c r="D160" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="D160" s="7" t="inlineStr">
+      <c r="E160" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3039,10 +3840,15 @@
           <t>Russia</t>
         </is>
       </c>
-      <c r="C161" s="6" t="n">
+      <c r="C161" s="11" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="D161" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="D161" s="7" t="inlineStr">
+      <c r="E161" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3057,10 +3863,15 @@
           <t>Zimbabwe</t>
         </is>
       </c>
-      <c r="C162" s="6" t="n">
+      <c r="C162" s="11" t="inlineStr">
+        <is>
+          <t>ZW</t>
+        </is>
+      </c>
+      <c r="D162" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="D162" s="7" t="inlineStr">
+      <c r="E162" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3075,10 +3886,15 @@
           <t>Guinea Bissau</t>
         </is>
       </c>
-      <c r="C163" s="6" t="n">
+      <c r="C163" s="11" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="D163" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="D163" s="7" t="inlineStr">
+      <c r="E163" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3093,10 +3909,15 @@
           <t>Mozambique</t>
         </is>
       </c>
-      <c r="C164" s="6" t="n">
+      <c r="C164" s="11" t="inlineStr">
+        <is>
+          <t>MZ</t>
+        </is>
+      </c>
+      <c r="D164" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="D164" s="7" t="inlineStr">
+      <c r="E164" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3111,10 +3932,15 @@
           <t>Cambodia</t>
         </is>
       </c>
-      <c r="C165" s="6" t="n">
+      <c r="C165" s="11" t="inlineStr">
+        <is>
+          <t>KH</t>
+        </is>
+      </c>
+      <c r="D165" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="D165" s="7" t="inlineStr">
+      <c r="E165" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3129,10 +3955,15 @@
           <t>Comoros</t>
         </is>
       </c>
-      <c r="C166" s="6" t="n">
+      <c r="C166" s="11" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="D166" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="D166" s="7" t="inlineStr">
+      <c r="E166" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3147,10 +3978,15 @@
           <t>Democratic Republic of the Congo</t>
         </is>
       </c>
-      <c r="C167" s="6" t="n">
+      <c r="C167" s="11" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="D167" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="D167" s="7" t="inlineStr">
+      <c r="E167" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3165,10 +4001,15 @@
           <t>Tajikistan</t>
         </is>
       </c>
-      <c r="C168" s="6" t="n">
+      <c r="C168" s="11" t="inlineStr">
+        <is>
+          <t>TJ</t>
+        </is>
+      </c>
+      <c r="D168" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="D168" s="7" t="inlineStr">
+      <c r="E168" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3183,10 +4024,15 @@
           <t>Burundi</t>
         </is>
       </c>
-      <c r="C169" s="6" t="n">
+      <c r="C169" s="11" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="D169" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="D169" s="7" t="inlineStr">
+      <c r="E169" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3201,10 +4047,15 @@
           <t>Turkmenistan</t>
         </is>
       </c>
-      <c r="C170" s="6" t="n">
+      <c r="C170" s="11" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="D170" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="D170" s="7" t="inlineStr">
+      <c r="E170" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3219,10 +4070,15 @@
           <t>Afghanistan</t>
         </is>
       </c>
-      <c r="C171" s="6" t="n">
+      <c r="C171" s="11" t="inlineStr">
+        <is>
+          <t>AF</t>
+        </is>
+      </c>
+      <c r="D171" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="D171" s="7" t="inlineStr">
+      <c r="E171" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3237,10 +4093,15 @@
           <t>Haiti</t>
         </is>
       </c>
-      <c r="C172" s="6" t="n">
+      <c r="C172" s="11" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+      <c r="D172" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="D172" s="7" t="inlineStr">
+      <c r="E172" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3255,10 +4116,15 @@
           <t>Myanmar</t>
         </is>
       </c>
-      <c r="C173" s="6" t="n">
+      <c r="C173" s="11" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="D173" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="D173" s="7" t="inlineStr">
+      <c r="E173" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3273,10 +4139,15 @@
           <t>Equatorial Guinea</t>
         </is>
       </c>
-      <c r="C174" s="6" t="n">
+      <c r="C174" s="11" t="inlineStr">
+        <is>
+          <t>GQ</t>
+        </is>
+      </c>
+      <c r="D174" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="D174" s="7" t="inlineStr">
+      <c r="E174" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3291,10 +4162,15 @@
           <t>Korea, North</t>
         </is>
       </c>
-      <c r="C175" s="6" t="n">
+      <c r="C175" s="11" t="inlineStr">
+        <is>
+          <t>KP</t>
+        </is>
+      </c>
+      <c r="D175" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="D175" s="7" t="inlineStr">
+      <c r="E175" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3309,10 +4185,15 @@
           <t>Syria</t>
         </is>
       </c>
-      <c r="C176" s="6" t="n">
+      <c r="C176" s="11" t="inlineStr">
+        <is>
+          <t>SY</t>
+        </is>
+      </c>
+      <c r="D176" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="D176" s="7" t="inlineStr">
+      <c r="E176" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3327,10 +4208,15 @@
           <t>Nicaragua</t>
         </is>
       </c>
-      <c r="C177" s="6" t="n">
+      <c r="C177" s="11" t="inlineStr">
+        <is>
+          <t>NI</t>
+        </is>
+      </c>
+      <c r="D177" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="D177" s="7" t="inlineStr">
+      <c r="E177" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3345,10 +4231,15 @@
           <t>Sudan</t>
         </is>
       </c>
-      <c r="C178" s="6" t="n">
+      <c r="C178" s="11" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="D178" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="D178" s="7" t="inlineStr">
+      <c r="E178" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3363,10 +4254,15 @@
           <t>Eritrea</t>
         </is>
       </c>
-      <c r="C179" s="6" t="n">
+      <c r="C179" s="11" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D179" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="D179" s="7" t="inlineStr">
+      <c r="E179" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3381,10 +4277,15 @@
           <t>Libya</t>
         </is>
       </c>
-      <c r="C180" s="6" t="n">
+      <c r="C180" s="11" t="inlineStr">
+        <is>
+          <t>LY</t>
+        </is>
+      </c>
+      <c r="D180" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="D180" s="7" t="inlineStr">
+      <c r="E180" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3399,10 +4300,15 @@
           <t>Yemen</t>
         </is>
       </c>
-      <c r="C181" s="6" t="n">
+      <c r="C181" s="11" t="inlineStr">
+        <is>
+          <t>YE</t>
+        </is>
+      </c>
+      <c r="D181" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="D181" s="7" t="inlineStr">
+      <c r="E181" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3417,10 +4323,15 @@
           <t>Venezuela</t>
         </is>
       </c>
-      <c r="C182" s="6" t="n">
+      <c r="C182" s="11" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="D182" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="D182" s="7" t="inlineStr">
+      <c r="E182" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3435,10 +4346,15 @@
           <t>Somalia</t>
         </is>
       </c>
-      <c r="C183" s="6" t="n">
+      <c r="C183" s="11" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="D183" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="D183" s="7" t="inlineStr">
+      <c r="E183" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3453,10 +4369,15 @@
           <t>South Sudan</t>
         </is>
       </c>
-      <c r="C184" s="6" t="n">
+      <c r="C184" s="11" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="D184" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="D184" s="7" t="inlineStr">
+      <c r="E184" s="7" t="inlineStr">
         <is>
           <t>高风险 High-risk</t>
         </is>
@@ -3464,7 +4385,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3476,11 +4397,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3501,6 +4423,11 @@
           <t>国家/地区 Country</t>
         </is>
       </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>代码 Code</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -3511,6 +4438,11 @@
           <t>Andorra</t>
         </is>
       </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -3521,6 +4453,11 @@
           <t>Anguilla</t>
         </is>
       </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -3531,6 +4468,11 @@
           <t>Antigua and Barbuda</t>
         </is>
       </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>AG</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -3541,6 +4483,11 @@
           <t>Aruba</t>
         </is>
       </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -3551,6 +4498,11 @@
           <t>Bahamas</t>
         </is>
       </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>BS</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -3561,6 +4513,11 @@
           <t>Bahrain</t>
         </is>
       </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>BH</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -3571,6 +4528,11 @@
           <t>Barbados</t>
         </is>
       </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -3581,6 +4543,11 @@
           <t>Belize</t>
         </is>
       </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>BZ</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -3591,6 +4558,11 @@
           <t>Bermuda</t>
         </is>
       </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>BM</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -3601,6 +4573,11 @@
           <t>Cayman Islands</t>
         </is>
       </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -3611,6 +4588,11 @@
           <t>Cook Islands</t>
         </is>
       </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -3621,6 +4603,11 @@
           <t>Curaçao</t>
         </is>
       </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>CW</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -3631,6 +4618,11 @@
           <t>Dominica</t>
         </is>
       </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -3641,6 +4633,11 @@
           <t>Gibraltar</t>
         </is>
       </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>GI</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -3651,6 +4648,11 @@
           <t>Grenada</t>
         </is>
       </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>GD</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -3661,6 +4663,11 @@
           <t>Guernsey</t>
         </is>
       </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>GG</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -3671,6 +4678,11 @@
           <t>Hong Kong</t>
         </is>
       </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -3681,6 +4693,11 @@
           <t>Isle of Man</t>
         </is>
       </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>IM</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -3691,6 +4708,11 @@
           <t>Jersey</t>
         </is>
       </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>JE</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -3701,6 +4723,11 @@
           <t>Lebanon</t>
         </is>
       </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -3711,6 +4738,11 @@
           <t>Liberia</t>
         </is>
       </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -3721,6 +4753,11 @@
           <t>Liechtenstein</t>
         </is>
       </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -3731,6 +4768,11 @@
           <t>Marshall Islands</t>
         </is>
       </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -3741,6 +4783,11 @@
           <t>Mauritius</t>
         </is>
       </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -3751,6 +4798,11 @@
           <t>Montserrat</t>
         </is>
       </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -3761,6 +4813,11 @@
           <t>Nauru</t>
         </is>
       </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -3771,6 +4828,11 @@
           <t>Niue</t>
         </is>
       </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -3781,6 +4843,11 @@
           <t>Panama</t>
         </is>
       </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -3791,6 +4858,11 @@
           <t>Philippines</t>
         </is>
       </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>PH</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -3801,6 +4873,11 @@
           <t>Saint Lucia</t>
         </is>
       </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>LC</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -3811,6 +4888,11 @@
           <t>Saint Vincent and the Grenadines</t>
         </is>
       </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -3821,6 +4903,11 @@
           <t>Samoa</t>
         </is>
       </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>AS</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -3831,6 +4918,11 @@
           <t>Seychelles</t>
         </is>
       </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -3841,6 +4933,11 @@
           <t>Singapore</t>
         </is>
       </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -3851,6 +4948,11 @@
           <t>Sint Maarten</t>
         </is>
       </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>SX</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -3861,6 +4963,11 @@
           <t>St Kitts and Nevis</t>
         </is>
       </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>KN</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -3871,6 +4978,11 @@
           <t>Turks and Caicos Islands</t>
         </is>
       </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -3881,6 +4993,11 @@
           <t>Vanuatu</t>
         </is>
       </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>VU</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -3891,6 +5008,11 @@
           <t>Virgin Islands (British)</t>
         </is>
       </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
@@ -3901,10 +5023,15 @@
           <t>Virgin Islands (U.S.)</t>
         </is>
       </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3916,12 +5043,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3942,7 +5069,12 @@
           <t>国家/地区 Country</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>代码 Code</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>含义</t>
         </is>
@@ -3959,7 +5091,12 @@
           <t>Democratic Republic of Korea</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>KP</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>严重战略缺陷：强化尽调，最严重者采取反制措施</t>
         </is>
@@ -3976,7 +5113,12 @@
           <t>Iran</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>IR</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>严重战略缺陷：强化尽调，最严重者采取反制措施</t>
         </is>
@@ -3993,7 +5135,12 @@
           <t>Myanmar</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>严重战略缺陷：强化尽调，最严重者采取反制措施</t>
         </is>
@@ -4010,7 +5157,12 @@
           <t>Angola</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>AO</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4027,7 +5179,12 @@
           <t>Bolivia</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>BO</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4044,7 +5201,12 @@
           <t>Bosnia and Herzegovina</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4061,7 +5223,12 @@
           <t>Bulgaria</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4078,7 +5245,12 @@
           <t>Cameroon</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4095,7 +5267,12 @@
           <t>Côte d'Ivoire</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4112,7 +5289,12 @@
           <t>Democratic Republic of the Congo</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4129,7 +5311,12 @@
           <t>Haiti</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4146,7 +5333,12 @@
           <t>Iraq</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>IQ</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4163,7 +5355,12 @@
           <t>Kenya</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>KE</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4180,7 +5377,12 @@
           <t>Kuwait</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>KW</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4197,7 +5399,12 @@
           <t>Lao PDR</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4214,7 +5421,12 @@
           <t>Lebanon</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4231,7 +5443,12 @@
           <t>Monaco</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4248,7 +5465,12 @@
           <t>Nepal</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4265,7 +5487,12 @@
           <t>Papua New Guinea</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4282,7 +5509,12 @@
           <t>South Sudan</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4299,7 +5531,12 @@
           <t>Syria</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>SY</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4316,7 +5553,12 @@
           <t>Venezuela</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4333,7 +5575,12 @@
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4350,7 +5597,12 @@
           <t>Virgin Islands (UK)</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>VG</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4367,7 +5619,12 @@
           <t>Yemen</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>YE</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>在 FATF 监督下整改中：加强监控</t>
         </is>
@@ -4375,7 +5632,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>